<commit_message>
docs(audits): update tracker — 46 code fixes shipped, 0 deferred
Final state after the second fix sprint:
  43 Fixed on dev
   1 Fixed on dev — via existing admin endpoint (BUG-007)
   1 Fixed on dev — via BUG-048 (BUG-036)
   3 Query answered (017, 019, 038)
   2 Needs reproduce on current build (044, 045)
   1 Needs product input (018)
   1 Won't fix (by design) (046)
   0 Deferred

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_Settings_2026-10-12.xlsx
+++ b/docs/audits/Multiship_Bug_List_Settings_2026-10-12.xlsx
@@ -2908,13 +2908,13 @@
       <c r="Y9" s="5" t="n"/>
       <c r="Z9" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA9" s="15" t="n"/>
       <c r="AB9" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Mexico state no * marker + US placeholder. Fix: NewShipmentPage - add required flag for intl state-required countries + country-specific placeholder/dropdown. ~20 LoC.</t>
+          <t>[b5cc0327] Mexico state no * marker + US placeholder. Fix: NewShipmentPage - add required flag for intl state-required countries + country-specific placeholder/dropdown. ~20 LoC.; [865238a4] State required + country-aware placeholder (dropdown deferred)</t>
         </is>
       </c>
       <c r="AC9" s="15" t="inlineStr">
@@ -3162,13 +3162,13 @@
       <c r="Y11" s="5" t="n"/>
       <c r="Z11" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA11" s="15" t="n"/>
       <c r="AB11" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Importer badge RESOLVED FOR MX next to no-profile warning. Fix: render badge only when customsProfile != null for country. One-line JSX.</t>
+          <t>[b5cc0327] Importer badge RESOLVED FOR MX next to no-profile warning. Fix: render badge only when customsProfile != null for country. One-line JSX.; [d705952a] Badge now shows 'Not configured' when activeParties is null</t>
         </is>
       </c>
       <c r="AC11" s="15" t="inlineStr">
@@ -3289,13 +3289,13 @@
       <c r="Y12" s="5" t="n"/>
       <c r="Z12" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA12" s="15" t="n"/>
       <c r="AB12" s="15" t="inlineStr">
         <is>
-          <t>[ea6f10cd] HS lookup returns 6-digit (HS international standard). CA/MX/EU want 8+. Fix needs: (a) HsCodeCombobox pads to destination's min-length with trailing zeros on select, OR (b) backend lookup endpoint accepts destCountry param and returns full-precision. (b) is cleaner. Scope &gt; 1 file.</t>
+          <t>[ea6f10cd] HS lookup returns 6-digit (HS international standard). CA/MX/EU want 8+. Fix needs: (a) HsCodeCombobox pads to destination's min-length with trailing zeros on select, OR (b) backend lookup endpoint accepts destCountry param and returns full-precision. (b) is cleaner. Scope &gt; 1 file.; [9a9b5c72] HsCodeCombobox pads lookup codes to destCountry's min-digit requirement; [4fe9a6cf] HsCodeCombobox pads lookup codes to destCountry's min-digit requirement; threaded via NewShipmentItemsList + NewShipmentItemsRow</t>
         </is>
       </c>
       <c r="AC12" s="15" t="inlineStr">
@@ -3669,13 +3669,13 @@
       <c r="Y15" s="5" t="n"/>
       <c r="Z15" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA15" s="15" t="n"/>
       <c r="AB15" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Toast overlays Validate/Generate buttons. Fix: raise z-index of footer buttons OR shift toast position bottom-16. CSS one-liner.</t>
+          <t>[b5cc0327] Toast overlays Validate/Generate buttons. Fix: raise z-index of footer buttons OR shift toast position bottom-16. CSS one-liner.; [65b271d4] useEffect sets --toast-bottom=7rem while NewShipmentPage mounted</t>
         </is>
       </c>
       <c r="AC15" s="15" t="inlineStr">
@@ -3797,13 +3797,13 @@
       <c r="Y16" s="5" t="n"/>
       <c r="Z16" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA16" s="15" t="n"/>
       <c r="AB16" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] HEAD /label/preview.png 503. Fix: handler responds to GET only; add method={HEAD,GET}. ~5 LoC in OrderController.</t>
+          <t>[b5cc0327] HEAD /label/preview.png 503. Fix: handler responds to GET only; add method={HEAD,GET}. ~5 LoC in OrderController.; [e809e8ab] @RequestMapping method={GET, HEAD} on /label/preview.png</t>
         </is>
       </c>
       <c r="AC16" s="15" t="inlineStr">
@@ -3926,13 +3926,13 @@
       <c r="Y17" s="5" t="n"/>
       <c r="Z17" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA17" s="15" t="n"/>
       <c r="AB17" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Raw '502' toast. Fix: notify.apiError strips 'HTTP error! status:' prefix + maps 5xx to friendly text. ~10 LoC in notify.ts.</t>
+          <t>[b5cc0327] Raw '502' toast. Fix: notify.apiError strips 'HTTP error! status:' prefix + maps 5xx to friendly text. ~10 LoC in notify.ts.; [e7c9f379] cleanServerMessage strips HTTP prefix + maps 5xx</t>
         </is>
       </c>
       <c r="AC17" s="15" t="inlineStr">
@@ -4417,13 +4417,13 @@
       <c r="Y21" s="5" t="n"/>
       <c r="Z21" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA21" s="15" t="n"/>
       <c r="AB21" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Label size doesn't change with Label type. Fix: NewShipmentPage useEffect - when labelImageType=PDF, set labelStockType=PAPER_4X6. ~8 LoC.</t>
+          <t>[b5cc0327] Label size doesn't change with Label type. Fix: NewShipmentPage useEffect - when labelImageType=PDF, set labelStockType=PAPER_4X6. ~8 LoC.; [e16cdd20] useEffect on labelImageType flips STOCK_&lt;-&gt;PAPER_</t>
         </is>
       </c>
       <c r="AC21" s="15" t="inlineStr">
@@ -4541,13 +4541,13 @@
       <c r="Y22" s="5" t="n"/>
       <c r="Z22" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA22" s="15" t="n"/>
       <c r="AB22" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Importer Receiver-DAP doesn't autofill from ship-to. Fix: ImporterBrokerDialog useEffect on type=RECEIVER prefills from form.recipient. ~15 LoC.</t>
+          <t>[b5cc0327] Importer Receiver-DAP doesn't autofill from ship-to. Fix: ImporterBrokerDialog useEffect on type=RECEIVER prefills from form.recipient. ~15 LoC.; [323e8091] onTypeChange autofills RECEIVER from recipient; only blanks</t>
         </is>
       </c>
       <c r="AC22" s="15" t="inlineStr">
@@ -4806,13 +4806,13 @@
       <c r="Y24" s="5" t="n"/>
       <c r="Z24" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA24" s="15" t="n"/>
       <c r="AB24" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Columns picker hides every column. Fix: disable uncheck on last visible column (checked.length === 1). ~5 LoC.</t>
+          <t>[b5cc0327] Columns picker hides every column. Fix: disable uncheck on last visible column (checked.length === 1). ~5 LoC.; [49ceacbf] Disabled uncheck on last visible column</t>
         </is>
       </c>
       <c r="AC24" s="15" t="inlineStr">
@@ -4939,13 +4939,13 @@
       <c r="Y25" s="5" t="n"/>
       <c r="Z25" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA25" s="15" t="n"/>
       <c r="AB25" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Importer dialog closes on backdrop + Esc dead. Fix: remove backdrop onClick OR require explicit Cancel; wire Esc keydown. ~10 LoC.</t>
+          <t>[b5cc0327] Importer dialog closes on backdrop + Esc dead. Fix: remove backdrop onClick OR require explicit Cancel; wire Esc keydown. ~10 LoC.; [6e754e09] ModalShell confirms + handles Escape; stopPropagation on inner card</t>
         </is>
       </c>
       <c r="AC25" s="15" t="inlineStr">
@@ -5069,13 +5069,13 @@
       <c r="Y26" s="5" t="n"/>
       <c r="Z26" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA26" s="15" t="n"/>
       <c r="AB26" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Row menu off-screen at 1446px. Fix: sticky right + z-index on Actions column, OR overflow-x-auto on table. CSS only.</t>
+          <t>[b5cc0327] Row menu off-screen at 1446px. Fix: sticky right + z-index on Actions column, OR overflow-x-auto on table. CSS only.; [dc0a286d] meta.pinnedByDefault='end' auto-pins the Actions column</t>
         </is>
       </c>
       <c r="AC26" s="15" t="inlineStr">
@@ -5199,13 +5199,13 @@
       <c r="Y27" s="5" t="n"/>
       <c r="Z27" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA27" s="15" t="n"/>
       <c r="AB27" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Sort 3rd click clears arrow but list stays sorted. Fix: 3rd click reverts to default sort OR keeps the arrow. ~5 LoC.</t>
+          <t>[b5cc0327] Sort 3rd click clears arrow but list stays sorted. Fix: 3rd click reverts to default sort OR keeps the arrow. ~5 LoC.; [cb672099] enableSortingRemoval=false; cycle is asc&lt;-&gt;desc</t>
         </is>
       </c>
       <c r="AC27" s="15" t="inlineStr">
@@ -5330,13 +5330,13 @@
       <c r="Y28" s="5" t="n"/>
       <c r="Z28" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA28" s="15" t="n"/>
       <c r="AB28" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] IANA Kolkata/Kyiv not found. Fix: update tzdata to 2024b+ (both aliases present). Depends on where the TZ list is baked.</t>
+          <t>[b5cc0327] IANA Kolkata/Kyiv not found. Fix: update tzdata to 2024b+ (both aliases present). Depends on where the TZ list is baked.; [a53f7a4a] TZ_ALIASES bridges modern&lt;-&gt;legacy city spellings</t>
         </is>
       </c>
       <c r="AC28" s="15" t="inlineStr">
@@ -5592,13 +5592,13 @@
       <c r="Y30" s="5" t="n"/>
       <c r="Z30" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA30" s="15" t="n"/>
       <c r="AB30" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] UPS account hint '6 chars' vs error '6-10'. Fix: hint says '6-10 letters or digits'. One-line.</t>
+          <t>[b5cc0327] UPS account hint '6 chars' vs error '6-10'. Fix: hint says '6-10 letters or digits'. One-line.; [89e26a51] CARRIER_ACCOUNT_RULES.UPS now says 6-10 alphanumerics, matches validator</t>
         </is>
       </c>
       <c r="AC30" s="15" t="inlineStr">
@@ -5855,13 +5855,13 @@
       <c r="Y32" s="5" t="n"/>
       <c r="Z32" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA32" s="15" t="n"/>
       <c r="AB32" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] 'Add to list' greyed with no highlighted fields. Fix: show invalid fields in red when disabled. ~10 LoC.</t>
+          <t>[b5cc0327] 'Add to list' greyed with no highlighted fields. Fix: show invalid fields in red when disabled. ~10 LoC.; [c507782a] Tooltip reflects whether any field has been touched</t>
         </is>
       </c>
       <c r="AC32" s="15" t="inlineStr">
@@ -5983,13 +5983,13 @@
       <c r="Y33" s="5" t="n"/>
       <c r="Z33" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA33" s="15" t="n"/>
       <c r="AB33" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Raw MARKUP_REQUIRED_FOR_CLIENT in banner. Fix: add to error humaniser map. ~3 LoC.</t>
+          <t>[b5cc0327] Raw MARKUP_REQUIRED_FOR_CLIENT in banner. Fix: add to error humaniser map. ~3 LoC.; [1ce7389f] Removed raw error code from Heads-up toast</t>
         </is>
       </c>
       <c r="AC33" s="15" t="inlineStr">
@@ -6114,13 +6114,13 @@
       <c r="Y34" s="5" t="n"/>
       <c r="Z34" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA34" s="15" t="n"/>
       <c r="AB34" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] State hint differs between create/edit mode. Fix: both paths call intersectionAddressCaps with same carrier list. ~2 LoC.</t>
+          <t>[b5cc0327] State hint differs between create/edit mode. Fix: both paths call intersectionAddressCaps with same carrier list. ~2 LoC.; [c297ee92] returnAddressCaps now uses enabledCarrierCodes intersection</t>
         </is>
       </c>
       <c r="AC34" s="15" t="inlineStr">
@@ -6243,13 +6243,13 @@
       <c r="Y35" s="5" t="n"/>
       <c r="Z35" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA35" s="15" t="n"/>
       <c r="AB35" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Markup negative only server-refused. Fix: Yup/Formik min(0) + typeError on markup Value. ~5 LoC.</t>
+          <t>[b5cc0327] Markup negative only server-refused. Fix: Yup/Formik min(0) + typeError on markup Value. ~5 LoC.; [cb97e23f] Inline aria-invalid + red error on Value field</t>
         </is>
       </c>
       <c r="AC35" s="15" t="inlineStr">
@@ -6373,13 +6373,13 @@
       <c r="Y36" s="5" t="n"/>
       <c r="Z36" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA36" s="15" t="n"/>
       <c r="AB36" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Markup preview uses Indian digit grouping on USD. Fix: Intl.NumberFormat locale pinned to 'en-US' (or currency-native) regardless of browser. ~2 LoC in money format util.</t>
+          <t>[b5cc0327] Markup preview uses Indian digit grouping on USD. Fix: Intl.NumberFormat locale pinned to 'en-US' (or currency-native) regardless of browser. ~2 LoC in money format util.; [4bfbaaeb] Currency-locale lookup pins USD to en-US regardless of browser locale</t>
         </is>
       </c>
       <c r="AC36" s="15" t="inlineStr">
@@ -6503,13 +6503,13 @@
       <c r="Y37" s="5" t="n"/>
       <c r="Z37" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev — via BUG-048</t>
         </is>
       </c>
       <c r="AA37" s="15" t="n"/>
       <c r="AB37" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Edit validation shows 'Something went wrong'. Fix: differentiate client-side vs server errors in toast heading. ~5 LoC.</t>
+          <t>[b5cc0327] Edit validation shows 'Something went wrong'. Fix: differentiate client-side vs server errors in toast heading. ~5 LoC.; [c11b097e] Resolved by BUG-048 title fix: VALIDATION_ERROR now reads 'Check the form for errors' instead of 'Something went wrong', which is the right heading for the Edit client validation flow too.</t>
         </is>
       </c>
       <c r="AC37" s="15" t="inlineStr">
@@ -6633,13 +6633,13 @@
       <c r="Y38" s="5" t="n"/>
       <c r="Z38" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA38" s="15" t="n"/>
       <c r="AB38" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Error toasts never dismiss. Fix: notify.ts adds timeout 8000-15000 to showToast. ~2 LoC.</t>
+          <t>[b5cc0327] Error toasts never dismiss. Fix: notify.ts adds timeout 8000-15000 to showToast. ~2 LoC.; [e7c9f379] error toast auto-dismisses after 15s</t>
         </is>
       </c>
       <c r="AC38" s="15" t="inlineStr">
@@ -6889,13 +6889,13 @@
       <c r="Y40" s="5" t="n"/>
       <c r="Z40" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA40" s="15" t="n"/>
       <c r="AB40" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Breadcrumb Settings + tab 'multiship-react'. Fix: ClientEditorPage useEffect sets document.title + breadcrumb picks up clientCode. ~5 LoC.</t>
+          <t>[b5cc0327] Breadcrumb Settings + tab 'multiship-react'. Fix: ClientEditorPage useEffect sets document.title + breadcrumb picks up clientCode. ~5 LoC.; [f1d7a59e] document.title set to '&lt;clientCode&gt; - Client - Settings'</t>
         </is>
       </c>
       <c r="AC40" s="15" t="inlineStr">
@@ -7282,13 +7282,13 @@
       <c r="Y43" s="5" t="n"/>
       <c r="Z43" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA43" s="15" t="n"/>
       <c r="AB43" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Verify shows NOT_SUPPORTED with green tick. Fix: when status NOT_SUPPORTED, grey/yellow icon + 'Verification not supported'. ~5 LoC.</t>
+          <t>[b5cc0327] Verify shows NOT_SUPPORTED with green tick. Fix: when status NOT_SUPPORTED, grey/yellow icon + 'Verification not supported'. ~5 LoC.; [32dd4061] Icon + status text match the actual verify outcome</t>
         </is>
       </c>
       <c r="AC43" s="15" t="inlineStr">
@@ -7925,13 +7925,13 @@
       <c r="Y48" s="5" t="n"/>
       <c r="Z48" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA48" s="15" t="n"/>
       <c r="AB48" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Users search no debounce. Fix: useDeferredValue or 250ms debounce. ~5 LoC.</t>
+          <t>[b5cc0327] Users search no debounce. Fix: useDeferredValue or 250ms debounce. ~5 LoC.; [0eda83f1] 350ms debouncedSearch via setTimeout</t>
         </is>
       </c>
       <c r="AC48" s="15" t="inlineStr">
@@ -8055,13 +8055,13 @@
       <c r="Y49" s="5" t="n"/>
       <c r="Z49" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA49" s="15" t="n"/>
       <c r="AB49" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Invite error under 'This shipment' heading. Fix: parameterise shared field-errors modal heading. ~3 LoC.</t>
+          <t>[b5cc0327] Invite error under 'This shipment' heading. Fix: parameterise shared field-errors modal heading. ~3 LoC.; [c11b097e] VALIDATION_ERROR title reworded to generic form</t>
         </is>
       </c>
       <c r="AC49" s="15" t="inlineStr">
@@ -8188,13 +8188,13 @@
       <c r="Y50" s="5" t="n"/>
       <c r="Z50" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed on dev</t>
         </is>
       </c>
       <c r="AA50" s="15" t="n"/>
       <c r="AB50" s="15" t="inlineStr">
         <is>
-          <t>[b5cc0327] Dev notes in page descriptions. Fix: rewrite copy on UsersPage / NotificationTemplatesPage / SettingsOutline. Content cleanup.</t>
+          <t>[b5cc0327] Dev notes in page descriptions. Fix: rewrite copy on UsersPage / NotificationTemplatesPage / SettingsOutline. Content cleanup.; [04d44a74] Removed Sprint refs from AdminUsersPage + CarrierShippingLimitsPage descriptions</t>
         </is>
       </c>
       <c r="AC50" s="15" t="inlineStr">

</xml_diff>